<commit_message>
feat: integrate rogue cards and commander updates
Add data-driven F4 card selection, layered comic artwork, randomized upgrade effects, model revisions, commander StateTree and navigation changes. Include the reusable card production skill and preserve prompt bytes; remove session scratch files.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeGameTexts.xlsx
+++ b/data/Excel/GuLiStrikeGameTexts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="464">
   <si>
     <t>文本id</t>
   </si>
@@ -1359,6 +1359,117 @@
   </si>
   <si>
     <t>延迟 {0} ms (RTT)</t>
+  </si>
+  <si>
+    <t>Card.WM01.FireRate.Title</t>
+  </si>
+  <si>
+    <t>战争机器肉鸽卡标题</t>
+  </si>
+  <si>
+    <t>增加射速</t>
+  </si>
+  <si>
+    <t>Card.WM01.FireRate.Description</t>
+  </si>
+  <si>
+    <t>战争机器肉鸽卡说明；{0}来自BonusPercent×100</t>
+  </si>
+  <si>
+    <t>战争机器的普攻射速提高 {0}%。</t>
+  </si>
+  <si>
+    <t>Card.WM01.HighSpeed.Title</t>
+  </si>
+  <si>
+    <t>极速机动</t>
+  </si>
+  <si>
+    <t>Card.WM01.HighSpeed.Description</t>
+  </si>
+  <si>
+    <t>战争机器的移动速度提高 {0}%。</t>
+  </si>
+  <si>
+    <t>Card.WM01.MissileDamage.Title</t>
+  </si>
+  <si>
+    <t>增加导弹伤害</t>
+  </si>
+  <si>
+    <t>Card.WM01.MissileDamage.Description</t>
+  </si>
+  <si>
+    <t>战争机器的导弹伤害提高 {0}%。</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Title</t>
+  </si>
+  <si>
+    <t>实战选牌界面</t>
+  </si>
+  <si>
+    <t>命运之选</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Entering</t>
+  </si>
+  <si>
+    <t>卡牌入场中…</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Choose</t>
+  </si>
+  <si>
+    <t>移动鼠标轻压牌面 · 单击选择 · Esc 取消</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Flip</t>
+  </si>
+  <si>
+    <t>翻牌中…</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Confirm</t>
+  </si>
+  <si>
+    <t>再次点击所选卡牌确认 · Esc 取消</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Submitting</t>
+  </si>
+  <si>
+    <t>正在确认加成…</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Success</t>
+  </si>
+  <si>
+    <t>加成已生效</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Failed</t>
+  </si>
+  <si>
+    <t>选牌失败：{0} · Esc 返回战场</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.OpenFailed</t>
+  </si>
+  <si>
+    <t>无法打开选牌：{0}</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Replay</t>
+  </si>
+  <si>
+    <t>重新播放</t>
+  </si>
+  <si>
+    <t>UI.RogueCards.Done</t>
+  </si>
+  <si>
+    <t>选择完成</t>
   </si>
 </sst>
 </file>
@@ -3819,6 +3930,193 @@
         <v>426</v>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="s">
+        <v>427</v>
+      </c>
+      <c r="B195" t="s">
+        <v>428</v>
+      </c>
+      <c r="C195" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="s">
+        <v>430</v>
+      </c>
+      <c r="B196" t="s">
+        <v>431</v>
+      </c>
+      <c r="C196" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="s">
+        <v>433</v>
+      </c>
+      <c r="B197" t="s">
+        <v>428</v>
+      </c>
+      <c r="C197" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="s">
+        <v>435</v>
+      </c>
+      <c r="B198" t="s">
+        <v>431</v>
+      </c>
+      <c r="C198" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="s">
+        <v>437</v>
+      </c>
+      <c r="B199" t="s">
+        <v>428</v>
+      </c>
+      <c r="C199" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="s">
+        <v>439</v>
+      </c>
+      <c r="B200" t="s">
+        <v>431</v>
+      </c>
+      <c r="C200" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="s">
+        <v>441</v>
+      </c>
+      <c r="B201" t="s">
+        <v>442</v>
+      </c>
+      <c r="C201" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="s">
+        <v>444</v>
+      </c>
+      <c r="B202" t="s">
+        <v>442</v>
+      </c>
+      <c r="C202" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="s">
+        <v>446</v>
+      </c>
+      <c r="B203" t="s">
+        <v>442</v>
+      </c>
+      <c r="C203" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="s">
+        <v>448</v>
+      </c>
+      <c r="B204" t="s">
+        <v>442</v>
+      </c>
+      <c r="C204" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="s">
+        <v>450</v>
+      </c>
+      <c r="B205" t="s">
+        <v>442</v>
+      </c>
+      <c r="C205" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="s">
+        <v>452</v>
+      </c>
+      <c r="B206" t="s">
+        <v>442</v>
+      </c>
+      <c r="C206" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="s">
+        <v>454</v>
+      </c>
+      <c r="B207" t="s">
+        <v>442</v>
+      </c>
+      <c r="C207" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="s">
+        <v>456</v>
+      </c>
+      <c r="B208" t="s">
+        <v>442</v>
+      </c>
+      <c r="C208" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="s">
+        <v>458</v>
+      </c>
+      <c r="B209" t="s">
+        <v>442</v>
+      </c>
+      <c r="C209" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="s">
+        <v>460</v>
+      </c>
+      <c r="B210" t="s">
+        <v>442</v>
+      </c>
+      <c r="C210" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="s">
+        <v>462</v>
+      </c>
+      <c r="B211" t="s">
+        <v>442</v>
+      </c>
+      <c r="C211" t="s">
+        <v>463</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: deliver PIE performance optimizations and threading plan
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeGameTexts.xlsx
+++ b/data/Excel/GuLiStrikeGameTexts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="567">
   <si>
     <t>文本id</t>
   </si>
@@ -1681,6 +1681,105 @@
   </si>
   <si>
     <t>彼之矛</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetThroughput</t>
+  </si>
+  <si>
+    <t>当前客户端连接实际累计字节差/真实秒；收+发合计；1KB=1000B，不是配置上限</t>
+  </si>
+  <si>
+    <t>网络 收 {0} KB/s | 发 {1} KB/s | 合计 {2} KB/s</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetPackets</t>
+  </si>
+  <si>
+    <t>当前连接包速率；丢包为UE计数差/秒，并非丢包百分比</t>
+  </si>
+  <si>
+    <t>包 收 {0}/s 发 {1}/s | 丢包 收 {2}/s 发 {3}/s</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetTransport</t>
+  </si>
+  <si>
+    <t>本端发送额度、所有通道可靠bunch待ACK数；欠账=max(QueuedBits,0)/8，非应用队列大小</t>
+  </si>
+  <si>
+    <t>本端额度 {0} KB/s | 可靠待确认 {1} 块 | 欠账 {2} KB</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetFlightReceive</t>
+  </si>
+  <si>
+    <t>解码飞行事件速率及应用载荷；不等于画面播放量；年龄用估计服务器时间，排除bootstrap，可能含时钟误差</t>
+  </si>
+  <si>
+    <t>飞行事件 收 {0}/s | 载荷 {1} KB/s | 平均估龄 {2} ms</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetPIETransport</t>
+  </si>
+  <si>
+    <t>同进程PIE匹配此客户端的服务器连接：下行发送额度、可靠待ACK块数和发送欠账</t>
+  </si>
+  <si>
+    <t>PIE下行额度 {0} KB/s | 可靠待确认 {1} 块 | 欠账 {2} KB</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetPIEFlightQueue</t>
+  </si>
+  <si>
+    <t>同进程PIE中此客户端的飞行应用队列；队首样本时间至服务器当前时间，不等于纯排队时间</t>
+  </si>
+  <si>
+    <t>PIE本连接 飞行待发 {0} 条 | 队首事件年龄 {1} ms</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetPending</t>
+  </si>
+  <si>
+    <t>新建或重连后先等待完整采样区间；未知值不能显示成零</t>
+  </si>
+  <si>
+    <t>网络 收 -- KB/s | 发 -- KB/s | 合计 -- KB/s</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetLocal</t>
+  </si>
+  <si>
+    <t>本面板按客户端ServerConnection统计，本地/服务端视口不显示其他客户端汇总</t>
+  </si>
+  <si>
+    <t>网络：本地视口（无客户端到服务器连接）</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetFlightPending</t>
+  </si>
+  <si>
+    <t>未得到连续两次飞行计数采样</t>
+  </si>
+  <si>
+    <t>飞行事件 收 --/s | 载荷 -- KB/s | 平均估龄 -- ms</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetPIEQueuePending</t>
+  </si>
+  <si>
+    <t>尚未建立此客户端的服务端飞行事件通道</t>
+  </si>
+  <si>
+    <t>PIE本连接 飞行待发 --（等待通道）</t>
+  </si>
+  <si>
+    <t>UI.Performance.NetPIEUnavailable</t>
+  </si>
+  <si>
+    <t>跨进程PIE或身份尚未匹配时，不产生额外RPC取得服务端信息</t>
+  </si>
+  <si>
+    <t>PIE服务端队列 --（需同进程服务端）</t>
   </si>
 </sst>
 </file>
@@ -4559,6 +4658,127 @@
         <v>533</v>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="s">
+        <v>534</v>
+      </c>
+      <c r="B233" t="s">
+        <v>535</v>
+      </c>
+      <c r="C233" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="s">
+        <v>537</v>
+      </c>
+      <c r="B234" t="s">
+        <v>538</v>
+      </c>
+      <c r="C234" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="s">
+        <v>540</v>
+      </c>
+      <c r="B235" t="s">
+        <v>541</v>
+      </c>
+      <c r="C235" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="s">
+        <v>543</v>
+      </c>
+      <c r="B236" t="s">
+        <v>544</v>
+      </c>
+      <c r="C236" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="s">
+        <v>546</v>
+      </c>
+      <c r="B237" t="s">
+        <v>547</v>
+      </c>
+      <c r="C237" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="s">
+        <v>549</v>
+      </c>
+      <c r="B238" t="s">
+        <v>550</v>
+      </c>
+      <c r="C238" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="s">
+        <v>552</v>
+      </c>
+      <c r="B239" t="s">
+        <v>553</v>
+      </c>
+      <c r="C239" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="s">
+        <v>555</v>
+      </c>
+      <c r="B240" t="s">
+        <v>556</v>
+      </c>
+      <c r="C240" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="s">
+        <v>558</v>
+      </c>
+      <c r="B241" t="s">
+        <v>559</v>
+      </c>
+      <c r="C241" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="s">
+        <v>561</v>
+      </c>
+      <c r="B242" t="s">
+        <v>562</v>
+      </c>
+      <c r="C242" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="s">
+        <v>564</v>
+      </c>
+      <c r="B243" t="s">
+        <v>565</v>
+      </c>
+      <c r="C243" t="s">
+        <v>566</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>